<commit_message>
[D1 D2] align received P0 contract and add verified dishwasher care sources
</commit_message>
<xml_diff>
--- a/data/research/r8-public-research-20261007/d1-d2-01a10600/reviews-238.xlsx
+++ b/data/research/r8-public-research-20261007/d1-d2-01a10600/reviews-238.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="Ra01917bcacd34a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="리뷰" sheetId="2" r:id="R9d18aa685f814e56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="관측" sheetId="3" r:id="R405db1bd2df4448e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제품·출처" sheetId="4" r:id="R5f62935e650a4849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="Rc1e1bd2d232342b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="리뷰" sheetId="2" r:id="R3d29677e92f8473c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="관측" sheetId="3" r:id="Rbf9e0ee18fca4afd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제품·출처" sheetId="4" r:id="Rc5dd34a982cd4024"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -780,7 +780,7 @@
       </x:c>
       <x:c r="B26" s="3"/>
       <x:c r="C26" s="3" t="str">
-        <x:v>PM P0 ResearchBundle 계약과 소비 인수는 미완료. 실제 모델 실행0회.</x:v>
+        <x:v>PM P0 계약 수신. 실행 입력3개 규격 검사 통과. 실제 모델 실행·서버 등록0회.</x:v>
       </x:c>
       <x:c r="D26" s="1"/>
     </x:row>
@@ -14952,7 +14952,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69e2774f2e054140"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re96916e7b4324556"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21248,7 +21248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7891a358385543e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b7b55b9bee74844"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23759,7 +23759,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9148b56df33b4d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca912edf0f77453c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>